<commit_message>
帯とタブの文字を IBM Plex Sans JP に変更 (version 0.4.6)
指示書の FONT を書体名で指定できるようにし、TP_GUIdocker_フォント フォルダの
書体を起動時にプラグイン内だけで読み込む。配布用の書体と許諾文書 (OFL) を dist に同梱。

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TP_GUIdocker_指示書.xlsx
+++ b/docs/TP_GUIdocker_指示書.xlsx
@@ -2483,7 +2483,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>FONT</t>
@@ -2491,15 +2491,19 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>タブ・ワークスペースの帯の文字</t>
+          <t>タブ・ワークスペースの帯の文字の書体</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>メニューバーと同じ</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr"/>
+          <t>IBM Plex Sans JP</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>書体</t>
+        </is>
+      </c>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -2508,7 +2512,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Windows がメニューに使う文字の種類と大きさ (帯の高さをメニューバーにそろえたため、最も自然に収まる)</t>
+          <t>書体名で指定 (「メニューバーと同じ」も可)。大きさはメニューバーの文字と同じ。パソコンに無い書体は、プラグインと同じ場所の「TP_GUIdocker_フォント」フォルダに置けば使える。見つからない時はメニューバーと同じ書体になる。候補の比較は docs/TP_GUIdocker_フォント比較.pdf</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4389,6 +4393,38 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>見た目</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>FONT</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>フォント比較の見本から IBM Plex Sans JP に決定</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>帯とタブの文字を IBM Plex Sans JP に変更し、書体名で指定できるようにした (書体はプラグインに同梱)</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>反映済み</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>